<commit_message>
fix: Either citizens or places of employment for matrix output
The construction of the `general_matrix_product` should not consider the
same array as selected by the `citizens_or_places_of_employment`
depending on the `citizens` flag. The threshold should rely on the
`places_of_employment` when `citizens = True` and on
`citizens_per_class` when `citizens = False`.
</commit_message>
<xml_diff>
--- a/tests/vlaanderen/reference/resultaten/werk/concurrentie/inwoners/restdag/Ontpl_concproduct_Auto.xlsx
+++ b/tests/vlaanderen/reference/resultaten/werk/concurrentie/inwoners/restdag/Ontpl_concproduct_Auto.xlsx
@@ -436,16 +436,16 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>460.370649390654</v>
+        <v>0</v>
       </c>
       <c r="C5">
-        <v>299.1221545791591</v>
+        <v>0</v>
       </c>
       <c r="D5">
-        <v>244.4989282820456</v>
+        <v>0</v>
       </c>
       <c r="E5">
-        <v>224.0371958427168</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -487,16 +487,16 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>2240.976194357066</v>
+        <v>0</v>
       </c>
       <c r="C8">
-        <v>1386.974704974449</v>
+        <v>0</v>
       </c>
       <c r="D8">
-        <v>1167.014165702147</v>
+        <v>0</v>
       </c>
       <c r="E8">
-        <v>1079.7131497476</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -521,16 +521,16 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>244.2138551302405</v>
+        <v>0</v>
       </c>
       <c r="C10">
-        <v>158.4617140933626</v>
+        <v>0</v>
       </c>
       <c r="D10">
-        <v>133.3524500112542</v>
+        <v>0</v>
       </c>
       <c r="E10">
-        <v>118.33617664089</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -538,16 +538,16 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>45.91022539218498</v>
+        <v>0</v>
       </c>
       <c r="C11">
-        <v>27.90136882217155</v>
+        <v>0</v>
       </c>
       <c r="D11">
-        <v>23.10162090392851</v>
+        <v>0</v>
       </c>
       <c r="E11">
-        <v>22.11439706454975</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -572,16 +572,16 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>136.1841753323431</v>
+        <v>0</v>
       </c>
       <c r="C13">
-        <v>88.01317346988841</v>
+        <v>0</v>
       </c>
       <c r="D13">
-        <v>74.91618632150265</v>
+        <v>0</v>
       </c>
       <c r="E13">
-        <v>67.28517365038661</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>